<commit_message>
Deploy 24/7 Cloud Serverless Webhook & Permanent Meta Token
</commit_message>
<xml_diff>
--- a/VENTA LIMPIA TU CLOSET.xlsx
+++ b/VENTA LIMPIA TU CLOSET.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30416"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30425"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5602c2dca830dca4/Documents/PROYECTO CON MONICA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="11_F25DC773A252ABDACC1048AAB1DD43425BDE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6852F86-8525-4508-A978-BFF44BB3BB84}"/>
+  <xr:revisionPtr revIDLastSave="106" documentId="11_F25DC773A252ABDACC1048AAB1DD43425BDE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6ADBB38-8014-4951-9C79-019F9E0BC660}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1590" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>NOMBRE</t>
   </si>
@@ -74,9 +74,6 @@
     <t>gaviotas juego</t>
   </si>
   <si>
-    <t>juego mandalas 3 piezas</t>
-  </si>
-  <si>
     <t>lampara monica</t>
   </si>
   <si>
@@ -114,6 +111,15 @@
   </si>
   <si>
     <t>COMISION</t>
+  </si>
+  <si>
+    <t>juego mandalas 3 piezas negro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 -150 </t>
+  </si>
+  <si>
+    <t>Cuadro Mariposas 80 X 120</t>
   </si>
 </sst>
 </file>
@@ -147,12 +153,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="6">
@@ -233,7 +245,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -250,9 +262,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -578,8 +593,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FC82F013-C7C9-4873-BA51-FB874FE75384}" name="Table1" displayName="Table1" ref="A1:I18" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" tableBorderDxfId="9" dataCellStyle="Currency">
-  <autoFilter ref="A1:I18" xr:uid="{FC82F013-C7C9-4873-BA51-FB874FE75384}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FC82F013-C7C9-4873-BA51-FB874FE75384}" name="Table1" displayName="Table1" ref="A1:I19" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" tableBorderDxfId="9" dataCellStyle="Currency">
+  <autoFilter ref="A1:I19" xr:uid="{FC82F013-C7C9-4873-BA51-FB874FE75384}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{B07B5AB9-1279-46E8-9DEE-546213F3DEE2}" name="NOMBRE" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{939F9481-9CD6-4FA6-A94C-5CBEC61FA4A2}" name="FECHA DE PUBLICACION" dataDxfId="7"/>
@@ -858,7 +873,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="50.6640625" customWidth="1"/>
@@ -877,28 +892,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -906,36 +921,38 @@
         <v>2</v>
       </c>
       <c r="B2" s="2"/>
-      <c r="C2" s="1"/>
+      <c r="C2" s="1">
+        <v>300</v>
+      </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="2"/>
       <c r="H2" s="1"/>
-      <c r="I2" s="12"/>
+      <c r="I2" s="11"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="14">
         <v>46261</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="15">
         <v>1000</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="15">
         <v>900</v>
       </c>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="2">
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="14">
         <v>46261</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="15">
         <v>900</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="15">
         <v>400</v>
       </c>
     </row>
@@ -944,7 +961,9 @@
         <v>4</v>
       </c>
       <c r="B4" s="2"/>
-      <c r="C4" s="1"/>
+      <c r="C4" s="1">
+        <v>80</v>
+      </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -957,7 +976,9 @@
         <v>5</v>
       </c>
       <c r="B5" s="2"/>
-      <c r="C5" s="1"/>
+      <c r="C5" s="1">
+        <v>500</v>
+      </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -987,7 +1008,9 @@
         <v>7</v>
       </c>
       <c r="B7" s="2"/>
-      <c r="C7" s="1"/>
+      <c r="C7" s="1">
+        <v>350</v>
+      </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -1000,7 +1023,9 @@
         <v>8</v>
       </c>
       <c r="B8" s="2"/>
-      <c r="C8" s="1"/>
+      <c r="C8" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -1013,7 +1038,9 @@
         <v>9</v>
       </c>
       <c r="B9" s="2"/>
-      <c r="C9" s="1"/>
+      <c r="C9" s="1">
+        <v>150</v>
+      </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
@@ -1026,7 +1053,9 @@
         <v>10</v>
       </c>
       <c r="B10" s="2"/>
-      <c r="C10" s="1"/>
+      <c r="C10" s="1">
+        <v>600</v>
+      </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
@@ -1039,7 +1068,9 @@
         <v>11</v>
       </c>
       <c r="B11" s="2"/>
-      <c r="C11" s="1"/>
+      <c r="C11" s="1">
+        <v>250</v>
+      </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
@@ -1049,10 +1080,12 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="B12" s="2"/>
-      <c r="C12" s="1"/>
+      <c r="C12" s="1">
+        <v>350</v>
+      </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
@@ -1062,10 +1095,12 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" s="2"/>
-      <c r="C13" s="1"/>
+      <c r="C13" s="1">
+        <v>350</v>
+      </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
@@ -1075,10 +1110,12 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" s="2"/>
-      <c r="C14" s="1"/>
+      <c r="C14" s="1">
+        <v>200</v>
+      </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
@@ -1088,10 +1125,12 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" s="2"/>
-      <c r="C15" s="1"/>
+      <c r="C15" s="1">
+        <v>250</v>
+      </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
@@ -1101,10 +1140,12 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16" s="2"/>
-      <c r="C16" s="1"/>
+      <c r="C16" s="1">
+        <v>1000</v>
+      </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -1114,10 +1155,12 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17" s="2"/>
-      <c r="C17" s="1"/>
+      <c r="C17" s="1">
+        <v>200</v>
+      </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
@@ -1127,10 +1170,12 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18" s="8"/>
-      <c r="C18" s="9"/>
+      <c r="C18" s="9">
+        <v>100</v>
+      </c>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
@@ -1139,15 +1184,30 @@
       <c r="I18" s="9"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="C19" s="10">
-        <f>SUM(C2:C18)</f>
-        <v>1600</v>
-      </c>
-      <c r="H19" s="11">
+      <c r="A19" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="1">
+        <v>500</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C20" s="12">
+        <f>SUM(C2:C19)</f>
+        <v>6780</v>
+      </c>
+      <c r="H20" s="10">
         <f>SUBTOTAL(109,Table1[PRECIO DE VENTA])</f>
         <v>900</v>
       </c>
-      <c r="I19" s="11">
+      <c r="I20" s="10">
         <f>SUBTOTAL(109,Table1[COMISION])</f>
         <v>400</v>
       </c>

</xml_diff>

<commit_message>
feat: fecha de publicacion en bot, vigencia automatica y orden cronologico descendente en chat
</commit_message>
<xml_diff>
--- a/VENTA LIMPIA TU CLOSET.xlsx
+++ b/VENTA LIMPIA TU CLOSET.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5602c2dca830dca4/Documents/PROYECTO CON MONICA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="106" documentId="11_F25DC773A252ABDACC1048AAB1DD43425BDE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6ADBB38-8014-4951-9C79-019F9E0BC660}"/>
+  <xr:revisionPtr revIDLastSave="188" documentId="11_F25DC773A252ABDACC1048AAB1DD43425BDE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF0E35D3-89F5-4E40-AC65-0DAC72F9C425}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28665" yWindow="-1605" windowWidth="29070" windowHeight="15750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>NOMBRE</t>
   </si>
@@ -120,6 +120,36 @@
   </si>
   <si>
     <t>Cuadro Mariposas 80 X 120</t>
+  </si>
+  <si>
+    <t>REPISA</t>
+  </si>
+  <si>
+    <t>PAQUETE PLATA RANCHO</t>
+  </si>
+  <si>
+    <t>AHORRO</t>
+  </si>
+  <si>
+    <t>total</t>
+  </si>
+  <si>
+    <t>sueldo Monica</t>
+  </si>
+  <si>
+    <t>Sueldo Kike</t>
+  </si>
+  <si>
+    <t>Ganancia</t>
+  </si>
+  <si>
+    <t>Gasto</t>
+  </si>
+  <si>
+    <t>Salidas</t>
+  </si>
+  <si>
+    <t>Dominio</t>
   </si>
 </sst>
 </file>
@@ -245,7 +275,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -264,16 +294,20 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="13">
     <dxf>
       <font>
         <b val="0"/>
@@ -291,6 +325,46 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -593,17 +667,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FC82F013-C7C9-4873-BA51-FB874FE75384}" name="Table1" displayName="Table1" ref="A1:I19" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" tableBorderDxfId="9" dataCellStyle="Currency">
-  <autoFilter ref="A1:I19" xr:uid="{FC82F013-C7C9-4873-BA51-FB874FE75384}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{B07B5AB9-1279-46E8-9DEE-546213F3DEE2}" name="NOMBRE" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{939F9481-9CD6-4FA6-A94C-5CBEC61FA4A2}" name="FECHA DE PUBLICACION" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{43C1CE85-C0BB-4D81-9904-9007022EB8BA}" name="PRECIO" dataDxfId="6" dataCellStyle="Currency"/>
-    <tableColumn id="4" xr3:uid="{4436F643-F567-49A6-81BF-223D7B646E93}" name="DESCUENTO 1" dataDxfId="5" dataCellStyle="Currency"/>
-    <tableColumn id="5" xr3:uid="{9042EB15-8319-47F4-894B-C5A67F7419EC}" name="DESCUENTO 2" dataDxfId="4" dataCellStyle="Currency"/>
-    <tableColumn id="6" xr3:uid="{ACD212E6-4DB2-46A8-8CB5-0CF691384FBC}" name="DESCUENTO 3 " dataDxfId="3" dataCellStyle="Currency"/>
-    <tableColumn id="7" xr3:uid="{9DAC8D39-CF3F-4123-B714-43F9BD3640EE}" name="FECHA DE VENTA" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{E2316F7E-D5BF-49CA-80C0-6B72480AEA68}" name="PRECIO DE VENTA" dataDxfId="1" dataCellStyle="Currency"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FC82F013-C7C9-4873-BA51-FB874FE75384}" name="Table1" displayName="Table1" ref="A1:J21" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11" tableBorderDxfId="10" dataCellStyle="Currency">
+  <autoFilter ref="A1:J21" xr:uid="{FC82F013-C7C9-4873-BA51-FB874FE75384}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{B07B5AB9-1279-46E8-9DEE-546213F3DEE2}" name="NOMBRE" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{939F9481-9CD6-4FA6-A94C-5CBEC61FA4A2}" name="FECHA DE PUBLICACION" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{43C1CE85-C0BB-4D81-9904-9007022EB8BA}" name="PRECIO" dataDxfId="7" dataCellStyle="Currency"/>
+    <tableColumn id="4" xr3:uid="{4436F643-F567-49A6-81BF-223D7B646E93}" name="DESCUENTO 1" dataDxfId="6" dataCellStyle="Currency"/>
+    <tableColumn id="5" xr3:uid="{9042EB15-8319-47F4-894B-C5A67F7419EC}" name="DESCUENTO 2" dataDxfId="5" dataCellStyle="Currency"/>
+    <tableColumn id="6" xr3:uid="{ACD212E6-4DB2-46A8-8CB5-0CF691384FBC}" name="DESCUENTO 3 " dataDxfId="4" dataCellStyle="Currency"/>
+    <tableColumn id="7" xr3:uid="{9DAC8D39-CF3F-4123-B714-43F9BD3640EE}" name="FECHA DE VENTA" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{E2316F7E-D5BF-49CA-80C0-6B72480AEA68}" name="PRECIO DE VENTA" dataDxfId="2" dataCellStyle="Currency"/>
+    <tableColumn id="10" xr3:uid="{9C420F7E-FAC2-4934-8C5B-2CD79E2C53B9}" name="AHORRO" dataDxfId="1" dataCellStyle="Currency"/>
     <tableColumn id="9" xr3:uid="{1E608A46-0E68-480C-9818-BCD5EE4F2C1B}" name="COMISION" dataDxfId="0" dataCellStyle="Currency"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -873,21 +948,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:V24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="50.6640625" customWidth="1"/>
-    <col min="2" max="2" width="14.44140625" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" customWidth="1"/>
+    <col min="1" max="1" width="34.33203125" customWidth="1"/>
+    <col min="2" max="2" width="13.77734375" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" customWidth="1"/>
     <col min="4" max="4" width="12.109375" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="12.109375" customWidth="1"/>
     <col min="7" max="7" width="13.109375" customWidth="1"/>
-    <col min="8" max="8" width="13.44140625" customWidth="1"/>
-    <col min="9" max="9" width="10.5546875" customWidth="1"/>
+    <col min="8" max="8" width="12.109375" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="10" width="10.5546875" customWidth="1"/>
+    <col min="12" max="12" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -913,10 +994,28 @@
         <v>23</v>
       </c>
       <c r="I1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L1" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="M1" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="N1" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="O1" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="P1" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
@@ -930,8 +1029,34 @@
       <c r="G2" s="2"/>
       <c r="H2" s="1"/>
       <c r="I2" s="11"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J2" s="11"/>
+      <c r="L2" s="12">
+        <f>H22</f>
+        <v>2800</v>
+      </c>
+      <c r="M2" s="10">
+        <f>L2*30%</f>
+        <v>840</v>
+      </c>
+      <c r="N2" s="10">
+        <f>L2*30%</f>
+        <v>840</v>
+      </c>
+      <c r="O2" s="10">
+        <f>L2*30%</f>
+        <v>840</v>
+      </c>
+      <c r="P2" s="10">
+        <f>L2*10%</f>
+        <v>280</v>
+      </c>
+      <c r="S2" s="12">
+        <f>500-N2</f>
+        <v>-340</v>
+      </c>
+      <c r="V2" s="12"/>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>3</v>
       </c>
@@ -953,10 +1078,16 @@
         <v>900</v>
       </c>
       <c r="I3" s="15">
+        <v>500</v>
+      </c>
+      <c r="J3" s="15">
         <v>400</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="O3">
+        <v>-200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>4</v>
       </c>
@@ -970,8 +1101,9 @@
       <c r="G4" s="2"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J4" s="1"/>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
@@ -985,8 +1117,9 @@
       <c r="G5" s="2"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>6</v>
       </c>
@@ -1002,8 +1135,9 @@
       <c r="G6" s="2"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J6" s="1"/>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
@@ -1017,8 +1151,9 @@
       <c r="G7" s="2"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J7" s="1"/>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>8</v>
       </c>
@@ -1032,8 +1167,9 @@
       <c r="G8" s="2"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J8" s="1"/>
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>9</v>
       </c>
@@ -1047,8 +1183,9 @@
       <c r="G9" s="2"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J9" s="1"/>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>10</v>
       </c>
@@ -1062,8 +1199,9 @@
       <c r="G10" s="2"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J10" s="1"/>
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>11</v>
       </c>
@@ -1077,8 +1215,13 @@
       <c r="G11" s="2"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J11" s="1"/>
+      <c r="S11">
+        <f>840-500+200</f>
+        <v>540</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>25</v>
       </c>
@@ -1092,8 +1235,9 @@
       <c r="G12" s="2"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J12" s="1"/>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>12</v>
       </c>
@@ -1107,8 +1251,9 @@
       <c r="G13" s="2"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J13" s="1"/>
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>13</v>
       </c>
@@ -1122,8 +1267,9 @@
       <c r="G14" s="2"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J14" s="1"/>
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>14</v>
       </c>
@@ -1137,8 +1283,9 @@
       <c r="G15" s="2"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J15" s="1"/>
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>15</v>
       </c>
@@ -1152,8 +1299,9 @@
       <c r="G16" s="2"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J16" s="1"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>16</v>
       </c>
@@ -1167,8 +1315,9 @@
       <c r="G17" s="2"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J17" s="1"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
         <v>17</v>
       </c>
@@ -1182,34 +1331,101 @@
       <c r="G18" s="8"/>
       <c r="H18" s="9"/>
       <c r="I18" s="9"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="6" t="s">
+      <c r="J18" s="9"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A19" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="B19" s="2"/>
-      <c r="C19" s="1">
+      <c r="B19" s="14"/>
+      <c r="C19" s="15">
         <v>500</v>
       </c>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="C20" s="12">
-        <f>SUM(C2:C19)</f>
-        <v>6780</v>
-      </c>
-      <c r="H20" s="10">
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="15">
+        <v>500</v>
+      </c>
+      <c r="I19" s="15">
+        <v>500</v>
+      </c>
+      <c r="J19" s="15"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A20" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" s="14"/>
+      <c r="C20" s="15">
+        <v>200</v>
+      </c>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="15">
+        <v>200</v>
+      </c>
+      <c r="I20" s="15">
+        <v>200</v>
+      </c>
+      <c r="J20" s="15"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A21" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="14"/>
+      <c r="C21" s="15">
+        <v>1200</v>
+      </c>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="15">
+        <v>1200</v>
+      </c>
+      <c r="I21" s="15">
+        <v>1200</v>
+      </c>
+      <c r="J21" s="16"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="C22" s="12">
+        <f>SUM(C2:C21)</f>
+        <v>8180</v>
+      </c>
+      <c r="H22" s="10">
         <f>SUBTOTAL(109,Table1[PRECIO DE VENTA])</f>
-        <v>900</v>
-      </c>
-      <c r="I20" s="10">
+        <v>2800</v>
+      </c>
+      <c r="I22" s="10">
+        <f>SUBTOTAL(109,Table1[AHORRO])</f>
+        <v>2400</v>
+      </c>
+      <c r="J22" s="10">
         <f>SUBTOTAL(109,Table1[COMISION])</f>
         <v>400</v>
+      </c>
+      <c r="O22" s="12">
+        <f>SUM(O2:O21)</f>
+        <v>640</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="10">
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: agregar soporte de enlace de Instagram en catalogo de ofertas y bot de WhatsApp
</commit_message>
<xml_diff>
--- a/VENTA LIMPIA TU CLOSET.xlsx
+++ b/VENTA LIMPIA TU CLOSET.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5602c2dca830dca4/Documents/PROYECTO CON MONICA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="188" documentId="11_F25DC773A252ABDACC1048AAB1DD43425BDE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF0E35D3-89F5-4E40-AC65-0DAC72F9C425}"/>
+  <xr:revisionPtr revIDLastSave="196" documentId="11_F25DC773A252ABDACC1048AAB1DD43425BDE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB46329C-56B7-4C8F-A801-BD91F7215A3E}"/>
   <bookViews>
-    <workbookView xWindow="28665" yWindow="-1605" windowWidth="29070" windowHeight="15750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>NOMBRE</t>
   </si>
@@ -150,6 +150,9 @@
   </si>
   <si>
     <t>Dominio</t>
+  </si>
+  <si>
+    <t>PAQUETE PLATA SHINO</t>
   </si>
 </sst>
 </file>
@@ -667,8 +670,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FC82F013-C7C9-4873-BA51-FB874FE75384}" name="Table1" displayName="Table1" ref="A1:J21" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11" tableBorderDxfId="10" dataCellStyle="Currency">
-  <autoFilter ref="A1:J21" xr:uid="{FC82F013-C7C9-4873-BA51-FB874FE75384}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FC82F013-C7C9-4873-BA51-FB874FE75384}" name="Table1" displayName="Table1" ref="A1:J22" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11" tableBorderDxfId="10" dataCellStyle="Currency">
+  <autoFilter ref="A1:J22" xr:uid="{FC82F013-C7C9-4873-BA51-FB874FE75384}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{B07B5AB9-1279-46E8-9DEE-546213F3DEE2}" name="NOMBRE" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{939F9481-9CD6-4FA6-A94C-5CBEC61FA4A2}" name="FECHA DE PUBLICACION" dataDxfId="8"/>
@@ -948,7 +951,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V24"/>
+  <dimension ref="A1:V25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34.33203125" customWidth="1"/>
@@ -962,6 +965,8 @@
     <col min="9" max="9" width="10" customWidth="1"/>
     <col min="10" max="10" width="10.5546875" customWidth="1"/>
     <col min="12" max="12" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11" customWidth="1"/>
+    <col min="14" max="14" width="11.21875" customWidth="1"/>
     <col min="15" max="15" width="10.21875" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="10.21875" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="9.44140625" bestFit="1" customWidth="1"/>
@@ -1031,7 +1036,7 @@
       <c r="I2" s="11"/>
       <c r="J2" s="11"/>
       <c r="L2" s="12">
-        <f>H22</f>
+        <f>H23</f>
         <v>2800</v>
       </c>
       <c r="M2" s="10">
@@ -1394,37 +1399,55 @@
       <c r="J21" s="16"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="C22" s="12">
-        <f>SUM(C2:C21)</f>
-        <v>8180</v>
-      </c>
-      <c r="H22" s="10">
-        <f>SUBTOTAL(109,Table1[PRECIO DE VENTA])</f>
-        <v>2800</v>
-      </c>
-      <c r="I22" s="10">
-        <f>SUBTOTAL(109,Table1[AHORRO])</f>
-        <v>2400</v>
-      </c>
-      <c r="J22" s="10">
-        <f>SUBTOTAL(109,Table1[COMISION])</f>
-        <v>400</v>
-      </c>
+      <c r="A22" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" s="14"/>
+      <c r="C22" s="15">
+        <v>1200</v>
+      </c>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="15">
+        <v>0</v>
+      </c>
+      <c r="I22" s="15"/>
+      <c r="J22" s="15"/>
       <c r="O22" s="12">
         <f>SUM(O2:O21)</f>
         <v>640</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>36</v>
+      <c r="C23" s="12">
+        <f>SUM(C2:C22)</f>
+        <v>9380</v>
+      </c>
+      <c r="H23" s="10">
+        <f>SUBTOTAL(109,Table1[PRECIO DE VENTA])</f>
+        <v>2800</v>
+      </c>
+      <c r="I23" s="10">
+        <f>SUBTOTAL(109,Table1[AHORRO])</f>
+        <v>2400</v>
+      </c>
+      <c r="J23" s="10">
+        <f>SUBTOTAL(109,Table1[COMISION])</f>
+        <v>400</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="10">
+      <c r="B25" s="10">
         <v>200</v>
       </c>
     </row>

</xml_diff>